<commit_message>
feat: add block assignment to bulk import
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -4,93 +4,77 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Trust-Wide Summary" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Alagar Kovil Registered Office" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Log - Alagar Kovil Registered O" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Aruldoss Puram Rehabilitation C" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Log - Aruldoss Puram Rehabilita" state="visible" r:id="rId8"/>
+    <sheet sheetId="1" name="Bulk Import Template" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="20">
-  <si>
-    <t>Metric</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Total Stock IN (This Month)</t>
-  </si>
-  <si>
-    <t>Total Stock OUT (This Month)</t>
-  </si>
-  <si>
-    <t>Total Current Stock (End of Month)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+  <si>
+    <t>Branch Name</t>
+  </si>
+  <si>
+    <t>Block</t>
   </si>
   <si>
     <t>Item Name</t>
   </si>
   <si>
-    <t>Quantity IN this month</t>
-  </si>
-  <si>
-    <t>Quantity OUT this month</t>
-  </si>
-  <si>
-    <t>Supplier/Party Name</t>
-  </si>
-  <si>
-    <t>Current Stock</t>
-  </si>
-  <si>
-    <t>first aid kit</t>
-  </si>
-  <si>
-    <t>Medico Pharmacy</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Movement Type</t>
-  </si>
-  <si>
-    <t>Quantity</t>
-  </si>
-  <si>
-    <t>Recorded By</t>
-  </si>
-  <si>
-    <t>2026-06-17</t>
-  </si>
-  <si>
-    <t>IN</t>
-  </si>
-  <si>
-    <t>admin@msctrust.org</t>
-  </si>
-  <si>
-    <t>2026-06-20</t>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>Initial Stock</t>
+  </si>
+  <si>
+    <t>Threshold</t>
+  </si>
+  <si>
+    <t>Unit Price</t>
+  </si>
+  <si>
+    <t>Item Code</t>
+  </si>
+  <si>
+    <t>Serial Number</t>
+  </si>
+  <si>
+    <t>Main Branch</t>
+  </si>
+  <si>
+    <t>Block A</t>
+  </si>
+  <si>
+    <t>Sample Item</t>
+  </si>
+  <si>
+    <t>Stationery</t>
+  </si>
+  <si>
+    <t>pcs</t>
+  </si>
+  <si>
+    <t>SKU-001</t>
+  </si>
+  <si>
+    <t>SN-123456789</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
       <scheme val="minor"/>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
     </font>
   </fonts>
   <fills count="2">
@@ -113,9 +97,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -455,261 +438,80 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="35" customWidth="1"/>
+    <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="5" max="8" width="15" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="10" max="10" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4">
-        <v>30</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="35" customWidth="1"/>
-    <col min="5" max="5" width="20" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
-      <c r="B2">
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2">
+        <v>100</v>
+      </c>
+      <c r="G2">
+        <v>10</v>
+      </c>
+      <c r="H2">
+        <v>50</v>
+      </c>
+      <c r="I2" t="s">
         <v>15</v>
       </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2">
-        <v>15</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="J2" t="s">
         <v>16</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D2">
-        <v>15</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="35" customWidth="1"/>
-    <col min="5" max="5" width="20" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2">
-        <v>15</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2">
-        <v>15</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D2">
-        <v>15</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>